<commit_message>
feat(excel-unprotect): implement streaming decryption and refine CLI experience
- Refactor Office file decryption to use a streaming, chunk-based approach, significantly reducing memory usage and improving robustness.
- Enhance interactive password input flow with retries and better error messaging.
- Improve temporary file cleanup logic, ensuring decrypted files are removed after processing.
- Update CLI tests to cover multi-sheet protection scenarios and verify temporary file removal.
- Optimize string allocations in path utility functions.
- Update `assert_cmd` and `predicates` dependencies.
- Remove unused `block-padding`, `byteorder`, `cbc`, and `regex` dependencies.
</commit_message>
<xml_diff>
--- a/crates/excel_unprotect/tests/fixtures/protected.xlsx
+++ b/crates/excel_unprotect/tests/fixtures/protected.xlsx
@@ -7,16 +7,24 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="MyProtectedSheet" sheetId="1" r:id="rId1"/>
+    <sheet name="MyUnprotectedSheet" sheetId="2" r:id="rId2"/>
+    <sheet name="AnotherProtected" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
-    <t>Protected Sheet</t>
+    <t>Locked</t>
+  </si>
+  <si>
+    <t>Open</t>
+  </si>
+  <si>
+    <t>LockedToo</t>
   </si>
 </sst>
 </file>
@@ -357,7 +365,38 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection password="83AF" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection password="CDA2" sheet="1" objects="1" scenarios="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection password="CDC2" sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>